<commit_message>
Revise Sugar News 2026-07-22 articles
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-22.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-22.xlsx
@@ -70,19 +70,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,12 +477,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
-  <cols>
-    <col width="55" customWidth="1" style="2" min="2" max="2"/>
-    <col width="55" customWidth="1" style="2" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -505,394 +497,360 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="180" customHeight="1" s="2">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>巴西</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ANTARA News报道：How sugarcane is powering Indonesias bioethanol ambition。来源：ANTARA News（https://news.google.com/rss/articles/CBMinwFBVV95cUxOS1YzTmlmWmFJT1pUYzZMTVZKVUtQUnYzQVhwN2Z1dFI0T3VNUXBaR2cxcFpxNDJqVmw3ejZtY1BIX1RNLUM4VjNtZmZlUzhBNUNHYlFGRk9Fbzh2NW9xaWtTa0hGcGFwdm1rbEh5czNQTEtCc3VhRGZkZ0prSTNaLVVlaFdHMzhUSF9zSlVxSG9yWnV5czBqQUN1dzRNUjTSAZ8BQVVfeXFMTktWM05pZlphSU9aVGM2TE1WSlVLUFJ2M0FYcDdmdXRSNE91TVFwWkdnMXBacTQyalZsN3o2bWNQSF9UTS1DOFYzbWZmZVM4QTVDR2JRRkZPRW84djVvcWlrU2tIRnBhcHZta2xIeXMzUExLQnN1YURmZGdKa0kzWi1VZWhXRzM4VEhfc0pVcUhvclp1eXMwakFDdXc0TVI0?oc=5）</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="180" customHeight="1" s="2">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>巴西</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 the-star.co.ke报道：Puzzle of tax-free Brazil sugar that originated from South Africa。来源：the-star.co.ke（https://news.google.com/rss/articles/CBMiugFBVV95cUxPa05kUGNibE8ydnd1NWpfRWNPMkZOMTBxQm54OUhla2FLYmJpUnpQUjRkN25LN3ZCbndMZlplT3pNZWNoZzFTQTFOVDd6OHU1RXI0SHg0MC03bjJuWUtSNnpPeU1JRjVYdDNVcFVlVEFZNWM1eU50ZldNWXNROWNJdlBHLWtYSU9ncC1VUUxBUDhrdlZFT042eU82OGpVOGlmc0t5UGtkUnBmaEtpU1RqZjc3dldKcmp5UkE?oc=5）</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="180" customHeight="1" s="2">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Valor International称，El Niño改善部分甘蔗产区单产，但降雨扰动也可能拖慢收割节奏。单产提升有利于增加糖料供应，收割延后则影响短期压榨节奏，综合影响暂偏中性。来源：Valor International（https://news.google.com/rss/articles/CBMiwwFBVV95cUxNRWt5MUNkWEJYejR0Q1lPaXd0WHlVcmhJVG5GM1J5ejBlV1Z6ZnkzeG1TSEFpSDg5clJPNklQV1RoRjNISE5uby1wNzVaeXNPTl9md3ZjSEVLTnJKMElUYTRhaTB6NG5nNFhLVGFLa0lfLWtkcm4xLXYwQnRjWkhSS01BNFpHOEJ0N3pGZVZzdTJJSVpHY05MNHVvVXZMdjhBd0dxMGdLSG9uQVNTTlYya21ld2ltc0lIV084eGZRX2Jua0nSAdIBQVVfeXFMUHJWYWRJMjlIYk1SbmU3cmxoVHpSZzM1NjNqS0wzWjJMaXRuRlNtTVBNZzBwaS02OHg0eVhwQXVLbzk0ZWw4UDZTOWdBVjR1aEV1aXhkTzlrcmU4cllwb0c0aGVLR25idTNLLV9QOElMQU93Xzl4RUlNbFJnUUdCdmtCMkxkMlZoQ3JYWkhMTmN2bUh4VmxyNXFWRkpMNFBrRkUzVUl1YWtReTZmMUdCSzNobE1hczF5VWlCcTVwTWNLUjhUVUYxcUNPM20wajM3bDlR?oc=5）</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>中性：单产和收割进度影响方向相反，短期对糖价缺乏单边驱动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 The Economic Times报道：Sugar stock limits may offer temporary relief but risk disrupting the supply chain: Industry。来源：The Economic Times（https://news.google.com/rss/articles/CBMihAJBVV95cUxPN3NiQ1g1OXUyc0JxT0hGZ2FQR2RtaEc3eGdJTzFkaGJmRXpYQ3NodmdlYkpfMXBmN2dGNXhtb096cVBVa29vNTU5V0R5Y1lTeFdMQnV1YjRlTk1HdnBCa2E5dno1SXdrbFlWSS00ZjdfazlWdnpnVVBFSkoxM1kxb0tjOC0yV1QxRXVnOGZZM0FpV0dRRzU4YXVZYVFUaWpLSFhZNzlzM0szZHJLNTRqTkpHSGVMb2F3Ry1SY1NBLWV6ZWpCSnhSM29iVVVMcE1ZV181LWdha0UzNDY4dWtkZmktcHpLUFcwMmRmZVd0dzBHdk5sa3BtNHFHdG1YOUc2UkhabtIBhAJBVV95cUxPN3NiQ1g1OXUyc0JxT0hGZ2FQR2RtaEc3eGdJTzFkaGJmRXpYQ3NodmdlYkpfMXBmN2dGNXhtb096cVBVa29vNTU5V0R5Y1lTeFdMQnV1YjRlTk1HdnBCa2E5dno1SXdrbFlWSS00ZjdfazlWdnpnVVBFSkoxM1kxb0tjOC0yV1QxRXVnOGZZM0FpV0dRRzU4YXVZYVFUaWpLSFhZNzlzM0szZHJLNTRqTkpHSGVMb2F3Ry1SY1NBLWV6ZWpCSnhSM29iVVVMcE1ZV181LWdha0UzNDY4dWtkZmktcHpLUFcwMmRmZVd0dzBHdk5sa3BtNHFHdG1YOUc2Ukhabg?oc=5）</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="180" customHeight="1" s="2">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>印度行业人士认为，食糖库存限制可在短期缓解价格压力，但可能扰乱糖厂、贸易商和终端之间的供应链安排。若监管加强，现货流通节奏可能放缓，但对总产量和库存水平的影响仍需观察。来源：The Economic Times（https://news.google.com/rss/articles/CBMihAJBVV95cUxPN3NiQ1g1OXUyc0JxT0hGZ2FQR2RtaEc3eGdJTzFkaGJmRXpYQ3NodmdlYkpfMXBmN2dGNXhtb096cVBVa29vNTU5V0R5Y1lTeFdMQnV1YjRlTk1HdnBCa2E5dno1SXdrbFlWSS00ZjdfazlWdnpnVVBFSkoxM1kxb0tjOC0yV1QxRXVnOGZZM0FpV0dRRzU4YXVZYVFUaWpLSFhZNzlzM0szZHJLNTRqTkpHSGVMb2F3Ry1SY1NBLWV6ZWpCSnhSM29iVVVMcE1ZV181LWdha0UzNDY4dWtkZmktcHpLUFcwMmRmZVd0dzBHdk5sa3BtNHFHdG1YOUc2UkhabtIBhAJBVV95cUxPN3NiQ1g1OXUyc0JxT0hGZ2FQR2RtaEc3eGdJTzFkaGJmRXpYQ3NodmdlYkpfMXBmN2dGNXhtb096cVBVa29vNTU5V0R5Y1lTeFdMQnV1YjRlTk1HdnBCa2E5dno1SXdrbFlWSS00ZjdfazlWdnpnVVBFSkoxM1kxb0tjOC0yV1QxRXVnOGZZM0FpV0dRRzU4YXVZYVFUaWpLSFhZNzlzM0szZHJLNTRqTkpHSGVMb2F3Ry1SY1NBLWV6ZWpCSnhSM29iVVVMcE1ZV181LWdha0UzNDY4dWtkZmktcHpLUFcwMmRmZVd0dzBHdk5sa3BtNHFHdG1YOUc2Ukhabg?oc=5）</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>中性：库存限制主要影响流通节奏，暂未改变印度食糖供需总量判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Revival of closed sugar mills, cane dues raised in Bihar Assembly。来源：ChiniMandi（https://news.google.com/rss/articles/CBMilwFBVV95cUxNY0t2TjlaYm94R2ZrcXU3T3paRlpSYjBxVVh4S0lhTWVZaDdPTGVaalgzSF96RHJmWEtkNXUwa1VyaGVMdXNGR2dFY0lYQmdBRTRHTmlJcFMtNmUyLW9temxNTFdnc25wdnVIMGRfTkNYTXJtWTZBcE51Y3NYcmJsa2FsYTZIajZmdmtXWktZR0pUaGtxLW1V?oc=5）</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="180" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>比哈尔邦议会讨论关闭糖厂重启和甘蔗款问题，地方政府继续关注糖厂运营和蔗农付款。若糖厂复产推进，将改善当地甘蔗消化能力，但短期尚未形成新增产量。来源：ChiniMandi（https://news.google.com/rss/articles/CBMilwFBVV95cUxNY0t2TjlaYm94R2ZrcXU3T3paRlpSYjBxVVh4S0lhTWVZaDdPTGVaalgzSF96RHJmWEtkNXUwa1VyaGVMdXNGR2dFY0lYQmdBRTRHTmlJcFMtNmUyLW9temxNTFdnc25wdnVIMGRfTkNYTXJtWTZBcE51Y3NYcmJsa2FsYTZIajZmdmtXWktZR0pUaGtxLW1V?oc=5）</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>中性：糖厂重启有利于中期加工能力恢复，短期对现货供应影响有限。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 Valor International报道：El Niño boosts sugarcane yields but may delay harvest。来源：Valor International（https://news.google.com/rss/articles/CBMiwwFBVV95cUxNRWt5MUNkWEJYejR0Q1lPaXd0WHlVcmhJVG5GM1J5ejBlV1Z6ZnkzeG1TSEFpSDg5clJPNklQV1RoRjNISE5uby1wNzVaeXNPTl9md3ZjSEVLTnJKMElUYTRhaTB6NG5nNFhLVGFLa0lfLWtkcm4xLXYwQnRjWkhSS01BNFpHOEJ0N3pGZVZzdTJJSVpHY05MNHVvVXZMdjhBd0dxMGdLSG9uQVNTTlYya21ld2ltc0lIV084eGZRX2Jua0nSAdIBQVVfeXFMUHJWYWRJMjlIYk1SbmU3cmxoVHpSZzM1NjNqS0wzWjJMaXRuRlNtTVBNZzBwaS02OHg0eVhwQXVLbzk0ZWw4UDZTOWdBVjR1aEV1aXhkTzlrcmU4cllwb0c0aGVLR25idTNLLV9QOElMQU93Xzl4RUlNbFJnUUdCdmtCMkxkMlZoQ3JYWkhMTmN2bUh4VmxyNXFWRkpMNFBrRkUzVUl1YWtReTZmMUdCSzNobE1hczF5VWlCcTVwTWNLUjhUVUYxcUNPM20wajM3bDlR?oc=5）</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="180" customHeight="1" s="2">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>印度政府在议会季风会议期间表示，糖厂已支付甘蔗款，且没有安排专项预算支持。甘蔗款支付改善有助于稳定蔗农现金流和后续种植积极性，对中长期糖料供应形成支撑。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirgFBVV95cUxQSXNzb2tRVzRBakhESjVETzJJYTFuTURoNFRpenl2V2REd2JkTDFZbWNYM1VhbGt1X2xmRHpNX25WTkgtcXJ5bGxwLXVlX0ZLYmIzcXBEaGZHTmRwWHl5aTFkbDZsWS1LZXpvcDN6cFU5ZUg4VWxianBJQ0NTd25teU9CRmIzd1hwSWszSVprcE45R1VXdlhrRFMwMFJzYnBGRnVJeW5PZ0dlbWU1Y1E?oc=5）</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>利空：甘蔗款支付改善有利于稳定未来糖料供应，方向上压制中长期糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Monsoon Session: Sugarcane dues paid by mills, no special budget support: Government。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirgFBVV95cUxQSXNzb2tRVzRBakhESjVETzJJYTFuTURoNFRpenl2V2REd2JkTDFZbWNYM1VhbGt1X2xmRHpNX25WTkgtcXJ5bGxwLXVlX0ZLYmIzcXBEaGZHTmRwWHl5aTFkbDZsWS1LZXpvcDN6cFU5ZUg4VWxianBJQ0NTd25teU9CRmIzd1hwSWszSVprcE45R1VXdlhrRFMwMFJzYnBGRnVJeW5PZ0dlbWU1Y1E?oc=5）</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>偏空糖价：生长阶段降雨增加有利于改善甘蔗水分条件和单产，可能增加未来糖料供应。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="180" customHeight="1" s="2">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>卡纳塔克邦甘蔗种植者要求全邦宣布干旱，并提出每英亩4万卢比救济诉求。若干旱影响持续，甘蔗生长和单产存在下修风险，可能削弱后续制糖原料供应。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiqwFBVV95cUxPb3pWb0dQMDZsR0tyamY2RUVscFAwdFplY21DcGs1ZEUzTWVBSTM1b1BtdEV6YjJ0VVplRUxaSEhYNVJtaXk0cnJBTGhvQ2tfOTlETm1BVTFTS1RIeVFrZHBHRzZJZnpqQmV0MWRQVzEyVjVvMmNlTDU4eF9JNWI2dGZWa2xzUlBFeUFiR0F6dTA4MkVvWVA0S0dRY2h3YndIS01pWC1rWWlISlE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>利多：干旱风险可能压低甘蔗单产和糖料供应，对糖价形成支撑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 DLH.net报道：Palm Sugar: A Village Story Launches on Windows PC on August 12。来源：DLH.net（https://news.google.com/rss/articles/CBMiowFBVV95cUxPelh6bGpuRTJSaUhyV3FsejVqdFFnaUVMVXdkbjVCZDBpVmctNDFUM2tRdWNtc2VTLTZ4blE3M2NPM2RkWjdzNDRKMkdhVnhfUERqUGdoTlFzcDJsNmVXRlRsRVVPNVduS3hoMDZlV0k4N0ZXT3JDVTc3TUdpVzgxMm9uU1ZUTGlFZWp6bXp0aUlMTzRqR1E4a3NWZWJqZ0lpWmtn?oc=5）</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="180" customHeight="1" s="2">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>印度政府表示，马哈拉施特拉邦甘蔗红腐病仍处于控制范围内。病害受控降低主产区减产风险，有利于稳定甘蔗供应和后续压榨预期。来源：ChiniMandi（https://news.google.com/rss/articles/CBMisgFBVV95cUxNdVVIbGlkZUJETHBGVGZOV0dkQTY5cGY3bWtHMGtlT2hJenVqOTR6cW0wNlkwRFpKSkpaTkFxNHBUTkpXejdORGpqdUYtZ29VLTYwM3NNVUtxMm15QXh3X2dlU2pLVWdsYm9lZjNfemxFdE0yRURId1RXTVpFdUxldUFYSHpJLVRKQ3hQVExhUk1RQk95d2xoTWptNWd0dVZUblk3eURZRmI1Z0JJTDRySmpB?oc=5）</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>利空：病害风险缓和有助于维持供应预期，对糖价偏利空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 BBC报道：22/07/26 Sugar beet factory closing, new Defra secretaryfarm fires, , oil seed rape harvest, hill farming in Wales。来源：BBC（https://news.google.com/rss/articles/CBMiUEFVX3lxTE53aXJVWlV3MGE5WEZJRHBhZE8tbm1JbnBvX21HZFJMeG1jaDhjckNBUVM1Q3BJc0VLMWVOcktFbERkbF9vRWlnUDgzdWdzS1lo?oc=5）</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="180" customHeight="1" s="2">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Moneycontrol指出，印度糖价上涨可能引发政策层面对市场秩序和价格稳定的关注。若监管进一步加强，可能通过销售配额、出口安排或乙醇分流政策影响糖厂经营，但当前仍以政策预期为主。来源：Moneycontrol.com（https://news.google.com/rss/articles/CBMiwAFBVV95cUxQakZ2UFZ3OUZ5a09ydnJueXM3OWRxcWtmcEFlLXd2SWlvWDV1MmZVV3dvVzBCTjlkUVlpaGpqLU03YmJ4YnJ5OVhqMk5nYVFpaTJtMWV3S3JmYVlGS0JuZE0wbUFPcFh4TkhoM1hLUVVpVUpMd1dUZTRxMC1DQkhud2NBeVlzLXpDTmltZE1LcW5rbHh1MGRBOG5VODQyQmtkMmE3X3kwRUJZMGRoc1pWQmplSVNxRXRHOG5meUhLeXDSAcABQVVfeXFMUGpGdlBWdzlGeWtPcnZybnlzNzlkcXFrZnBBZS13dklpb1g1dTJmVVd3b1cwQk45ZFFZaWhqai1NN2JieGJyeTlYajJOZ2FRaWkybTFld0tyZmFZRktCbmRNMG1BT3BYeE5IaDNYS1FVaVVKTHdXVGU0cTAtQ0JIbndjQXlZcy16Q05pbWRNS3Fua2x4dTBkQThuVTg0MkJrZDJhN195MEVCWTBkaHNaVkJqZUlTcUV0RzhuZnlIS3lw?oc=5）</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>中性：价格上涨带来监管风险，但尚未形成明确供需调整措施。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 indiagazette.com报道：Bengaluru-Based Author Akoparna B Debuts with Emotionally Powerful Novel The Burnt Sugar Club。来源：indiagazette.com（https://news.google.com/rss/articles/CBMi0wFBVV95cUxNN3pNQzU5a1JucU9nN3N5RkpiWEZwMnl1c3N0U050TTJCLWRzLWNMZG5VSGRVWUdyR1hBajhSVXZpM01nWFNjT09pMXpodGJFdGpNb0gzLUJfN01RRGp2Ml9fbGxrcW9yY0xCb3JvcEFmRV9TUExYMkJ5RFBuZDNXNXhUVktvTmRxSV9IOHdmQlU0MDdjdEdCU1MyYl96VzJVTWhUVVRNTWhWNEd1TnFQVm9iMDU0cTNVSFVrSy1INExuLWF1cnBvenlkbzhDa1Mta0J3?oc=5）</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="180" customHeight="1" s="2">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 FBC News报道：Labour shortage slows sugar production。来源：FBC News（https://news.google.com/rss/articles/CBMie0FVX3lxTE9pckZqdmNDanNIakl6SkR2SkZLVWxmREhfNWF6elE2U3YyUG1OQWtGc19CWExiZnJPcURlUWxTS0M3d2ZKdnJFM3E1TENKWE5rTkJYOHhibG5ZRDdDRHBucUVzYUhUUi1MOGNncXNkNXFCdkJCeWtRVm5YZw?oc=5）</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>偏多糖价：贸易限制或供应扰动可能减少国际市场可用糖源。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="180" customHeight="1" s="2">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Karnataka sugarcane growers seek state-wide drought declaration, Rs 40,000 relief。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiqwFBVV95cUxPb3pWb0dQMDZsR0tyamY2RUVscFAwdFplY21DcGs1ZEUzTWVBSTM1b1BtdEV6YjJ0VVplRUxaSEhYNVJtaXk0cnJBTGhvQ2tfOTlETm1BVTFTS1RIeVFrZHBHRzZJZnpqQmV0MWRQVzEyVjVvMmNlTDU4eF9JNWI2dGZWa2xzUlBFeUFiR0F6dTA4MkVvWVA0S0dRY2h3YndIS01pWC1rWWlISlE?oc=5）</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="180" customHeight="1" s="2">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Monsoon Session: Red Rot disease remains under control in Maharashtra, Government says。来源：ChiniMandi（https://news.google.com/rss/articles/CBMisgFBVV95cUxNdVVIbGlkZUJETHBGVGZOV0dkQTY5cGY3bWtHMGtlT2hJenVqOTR6cW0wNlkwRFpKSkpaTkFxNHBUTkpXejdORGpqdUYtZ29VLTYwM3NNVUtxMm15QXh3X2dlU2pLVWdsYm9lZjNfemxFdE0yRURId1RXTVpFdUxldUFYSHpJLVRKQ3hQVExhUk1RQk95d2xoTWptNWd0dVZUblk3eURZRmI1Z0JJTDRySmpB?oc=5）</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>偏空糖价：生长阶段降雨增加有利于改善甘蔗水分条件和单产，可能增加未来糖料供应。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="180" customHeight="1" s="2">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 Barchart.com报道：Rising Crude Oil Prices Support Sugar。来源：Barchart.com（https://news.google.com/rss/articles/CBMiiAFBVV95cUxQZWFVUFdFYWVLRnlON2YxV2N5YTVKMDdsNFkxVnUtVG5IOHpOMkhDb2xyVTc0TlZlTnIyRm5SV19FU0p2MGFyLTRhVDZFSFN1TFg2bHAySG9hQkFVVjgweGxFLUNnWVJjMWZOa2RDZmVidmVidERiZ1FrakpkaE9mVFlxbnZLa0Zo?oc=5）</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="180" customHeight="1" s="2">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>印度</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 Moneycontrol.com报道：Chart of the Day | Sugar price rise may invite unwanted attention。来源：Moneycontrol.com（https://news.google.com/rss/articles/CBMiwAFBVV95cUxQakZ2UFZ3OUZ5a09ydnJueXM3OWRxcWtmcEFlLXd2SWlvWDV1MmZVV3dvVzBCTjlkUVlpaGpqLU03YmJ4YnJ5OVhqMk5nYVFpaTJtMWV3S3JmYVlGS0JuZE0wbUFPcFh4TkhoM1hLUVVpVUpMd1dUZTRxMC1DQkhud2NBeVlzLXpDTmltZE1LcW5rbHh1MGRBOG5VODQyQmtkMmE3X3kwRUJZMGRoc1pWQmplSVNxRXRHOG5meUhLeXDSAcABQVVfeXFMUGpGdlBWdzlGeWtPcnZybnlzNzlkcXFrZnBBZS13dklpb1g1dTJmVVd3b1cwQk45ZFFZaWhqai1NN2JieGJyeTlYajJOZ2FRaWkybTFld0tyZmFZRktCbmRNMG1BT3BYeE5IaDNYS1FVaVVKTHdXVGU0cTAtQ0JIbndjQXlZcy16Q05pbWRNS3Fua2x4dTBkQThuVTg0MkJrZDJhN195MEVCWTBkaHNaVkJqZUlTcUV0RzhuZnlIS3lw?oc=5）</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="180" customHeight="1" s="2">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 Whalesbook报道：Sugar Price Hike Triggers Government Call to Curb Hoarding。来源：Whalesbook（https://news.google.com/rss/articles/CBMi0AFBVV95cUxNbGhqTllSVU9KdDh0MnVTRnVEU05zU1BsT2FYVEVHUUVyZHo2eVZLOTFmMU9pNGU3VVFrUUNOVTBzbWI3a0hBZEQwRWFLTllacGFUMHFRUlhZdmI3QVllbFZTcklKQWtDZklBbXpMZFUyLXYteWl5UGR4TUdTTWNnc2xRNFlfU2VmRjVKUlpJM0tlUjFvYUMtTjdLdzI0MW1vam85VlJDcUhId1IyMGtTUTV2TllLMDg1LUpRN29ISXNWV2pwTFFBdnp2eENINVhl?oc=5）</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="180" customHeight="1" s="2">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Poland proposes higher sugar tax, industry warns of impact on food and beverage sector。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiswFBVV95cUxOd1QyWVNpQ0FJSkFBSk55NWh1b0pyQzI0NGFGaU5LWGhXSWhlYU16LTdEdnRwM05XVldFNmx2NjV4aFNKeTJ0WHo0cGVqQmJnMUZuXzFfOUpFb1VRckd2Q3VjbDlBaVVXaHl5b19pWEZ6ODhMNGF1LU5aazJjSEFGWk1nektIbGt4SXFxSTFlUXFYWEpEbm9ubWJ5NVJaUkxVOVczU1VxWF9SQko1Mi15ckZiZw?oc=5）</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="180" customHeight="1" s="2">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>印度糖价上涨后，政府要求行业抑制囤货和投机，以维持节日期间零售价格稳定。行业承诺推动新榨季提前开榨，若落实将增加国内供应节奏并抑制现货涨幅。来源：Whalesbook（https://news.google.com/rss/articles/CBMi0AFBVV95cUxNbGhqTllSVU9KdDh0MnVTRnVEU05zU1BsT2FYVEVHUUVyZHo2eVZLOTFmMU9pNGU3VVFrUUNOVTBzbWI3a0hBZEQwRWFLTllacGFUMHFRUlhZdmI3QVllbFZTcklKQWtDZklBbXpMZFUyLXYteWl5UGR4TUdTTWNnc2xRNFlfU2VmRjVKUlpJM0tlUjFvYUMtTjdLdzI0MW1vam85VlJDcUhId1IyMGtTUTV2TllLMDg1LUpRN29ISXNWV2pwTFFBdnp2eENINVhl?oc=5）</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>利空：抑制囤货和提前开榨有助于增加市场供应，对印度糖价偏利空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>英国</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 Food and Drink International报道：British Sugar proposes closure of Cantley factory to support competitiveness。来源：Food and Drink International（https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR01lb3dWYnZCc0tKWkd5OE42ZjlKa3owRy04ZTA3ZThUcmNid3FmeTd2d0t3N1dXYmQxX0dXcnJjYXo5WmJGd1ctQ3lKZXhtMndYVHhkMkE1YXVWUmZNWEpIZUtYSDBfYmNQZ004bm9jV1JlMW1IWkswa01ralA3eHZ3N0wzZUVhUmhCYkxHNEFCSEMwWFVwT2FBallSZGhGZlY2aXBGTGNkMW5MQVVWclNfQmJEbnFf?oc=5）</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="180" customHeight="1" s="2">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>BBC节目涉及英国甜菜糖厂关闭及农业政策调整，显示英国甜菜糖加工布局继续收缩。相关影响取决于替代工厂承接能力，短期对国内食糖供应仍需跟踪。来源：BBC（https://news.google.com/rss/articles/CBMiUEFVX3lxTE53aXJVWlV3MGE5WEZJRHBhZE8tbm1JbnBvX21HZFJMeG1jaDhjckNBUVM1Q3BJc0VLMWVOcktFbERkbF9vRWlnUDgzdWdzS1lo?oc=5）</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>中性：单厂调整影响区域甜菜消化，但全国供应影响尚不明确。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>英国</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：British sugar proposes closure of historic Cantley factory, over 100 jobs at risk。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirAFBVV95cUxObnJJb1pyWU5hbnVUMVBZNHV0MVZ5akZQLTB5RU96OVBkZnhJaEdmV1VyMlY4ZndmTlBBRXB0NFY1bUVScF80YkxUWWhNR1hHWmpLNXFmYndDc1hZTk9IeUk2aEhNYVdkOWsxN2VVTVd1SWVrWDZqOUlEWGdJS3dOR0x4NG5iNDhoRDRoSjJIUmF4a3dIT0hwR3hTVG02UzNrX2xaQ1NHUndTT3VS?oc=5）</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="180" customHeight="1" s="2">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 UkrAgroConsult报道：Poland’s sugar production could fall by 17%。来源：UkrAgroConsult（https://news.google.com/rss/articles/CBMigwFBVV95cUxNRmgyRnZoMWIyTEUtLUFjS2padHhNR0tuZDE5T0pGTzZLUWlxS1lNQloxaFFUaUpWNW41UEJRUU9RZmR2NUxwY3ViQmx0SVM5cklFM2NHUEt3cUpvekpSM2g1ME1jYXBqZVoza2p4NXphcEFiZlY3Q0hmaVlGRU9xU29DQQ?oc=5）</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="180" customHeight="1" s="2">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ABC7 Bay Area报道：C&amp;H Sugar strike: Arrests, injuries reported at strike line in Crockett。来源：ABC7 Bay Area（https://news.google.com/rss/articles/CBMilgFBVV95cUxQY2x4cG8yOGF1NTQ3eVBUVW9JRVkzQXBxR25pVEhxRm95UFBEMV9BdEZoVXVocC1uQ0c5TzlmTzREdzRKWUtVbXJQX29zVEY3QkI0TzVCSWktMHRhUE9abU45SlVCVnhzSmdQUkFnMzBpZUtNUUE1eWNSbGVqT01LUkVjb1ZsZ3QteEE2eUR1NV9HLWY2TlHSAZsBQVVfeXFMT0w1bk1yajBVSVp0dlBmMEJOZXlHMUQ5WHgzSEpnYTZack1FVUtsTVYwS2c4TGN0TWtsWktTcjlIemFDTW1OZFNoLUhPcGxWQlJZMGdzVXRjdzBKWVhjZGk5bXMyd01Dd3RXMjJ4R3pwMnNDLWZ2SmVNTjNGUkpGLVg0cWUxTVRpN0pib1lFUUJ3bElLNGU1aDRnWFE?oc=5）</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="180" customHeight="1" s="2">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 The Telegraph报道：Britain’s oldest sugar factory shuts because of sky-high energy costs。来源：The Telegraph（https://news.google.com/rss/articles/CBMiqgFBVV95cUxOa2xFWmhEQmg2M29sUnduS2RtMG41TFJCVDNBNFRuamF2d1NBV09ndGtMLWhnS0dmbXM2eXBNMzJGWE5nTFZtNEJDZjNDbVRNLWk5VzVhc1BiWDlHQXdjTmdZWHVBOGVnQldPcG1PeUVlcTRSZXZjSXExR3phbFVxRlZ3SzI2amtEcEN5aEZnQlZWMTNibXpQVU5vUGhOU2tmTGpNQ3BrSVF6UQ?oc=5）</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="180" customHeight="1" s="2">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>其他国家</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 czapp.com报道：Higher Sugar Content Offsets Slow Start to Queensland Harvest。来源：czapp.com（https://news.google.com/rss/articles/CBMiowFBVV95cUxQcVd5RDJSRzJQX3RzdkhSa2k3TndUSDREUGludzZmaTRlZG1JQ1FxSlNqTzRuc3pSSlVfRk16dTFvOVZtYVpUUFc2aXR1X3A2X3o2RzU3Ul9SODJPdEdMbjlTS2FIMUlnZ1hHM18tTjdTNlVVQU5VWE9PTVNaV1k0S3JSQjAyMnZzYnlZckZmZkxSRnJHUzhQbjdVZ1V4SWFjRlFj?oc=5）</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="180" customHeight="1" s="2">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The Telegraph称，英国历史最久的糖厂因高能源成本关闭。能源成本上升压缩甜菜糖加工利润，若产能退出落地，可能削弱英国本土制糖能力。来源：The Telegraph（https://news.google.com/rss/articles/CBMiqgFBVV95cUxOa2xFWmhEQmg2M29sUnduS2RtMG41TFJCVDNBNFRuamF2d1NBV09ndGtMLWhnS0dmbXM2eXBNMzJGWE5nTFZtNEJDZjNDbVRNLWk5VzVhc1BiWDlHQXdjTmdZWHVBOGVnQldPcG1PeUVlcTRSZXZjSXExR3phbFVxRlZ3SzI2amtEcEN5aEZnQlZWMTNibXpQVU5vUGhOU2tmTGpNQ3BrSVF6UQ?oc=5）</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>利多：加工产能退出和成本压力可能收缩本土供应，对糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>British Sugar计划关闭Cantley工厂，以提升公司竞争力和运营效率。该调整反映英国甜菜糖行业成本和产能布局压力，但短期供应影响取决于其他工厂承接情况。来源：Food and Drink International（https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR01lb3dWYnZCc0tKWkd5OE42ZjlKa3owRy04ZTA3ZThUcmNid3FmeTd2d0t3N1dXYmQxX0dXcnJjYXo5WmJGd1ctQ3lKZXhtMndYVHhkMkE1YXVWUmZNWEpIZUtYSDBfYmNQZ004bm9jV1JlMW1IWkswa01ralA3eHZ3N0wzZUVhUmhCYkxHNEFCSEMwWFVwT2FBallSZGhGZlY2aXBGTGNkMW5MQVVWclNfQmJEbnFf?oc=5）</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>中性：产能整合改善企业效率，但对当期供应的影响尚待确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ChiniMandi称，British Sugar拟关闭历史悠久的Cantley工厂，超过100个岗位面临风险。若关闭执行，将减少当地甜菜加工节点，对区域甜菜收购和制糖能力构成压力。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirAFBVV95cUxObnJJb1pyWU5hbnVUMVBZNHV0MVZ5akZQLTB5RU96OVBkZnhJaEdmV1VyMlY4ZndmTlBBRXB0NFY1bUVScF80YkxUWWhNR1hHWmpLNXFmYndDc1hZTk9IeUk2aEhNYVdkOWsxN2VVTVd1SWVrWDZqOUlEWGdJS3dOR0x4NG5iNDhoRDRoSjJIUmF4a3dIT0hwR3hTVG02UzNrX2xaQ1NHUndTT3VS?oc=5）</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>利多：区域加工能力下降可能削弱本土糖源供给，对糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>斐济</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-22 ChiniMandi报道：Fiji: Labour shortage slows cane harvesting。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiekFVX3lxTFBEUUY2QWU3MmxCcjZHcGwzM2phb1gwaG5PRFJEUUFGYVBwRnBjT0lxNzZudk9aODB6MGMzcm9pczNiYmlSbDdTUm5ucUdZTm1HOUFRbWhhazhVYXlvZDNER2NfWkdzb200WDlGY2ZlLUJ6MDdGMktxc2RR?oc=5）</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>偏多糖价：贸易限制或供应扰动可能减少国际市场可用糖源。</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>FBC News称，斐济劳动力短缺拖慢食糖生产。采收和压榨环节受限可能影响甘蔗入榨进度，增加当期产糖不确定性。来源：FBC News（https://news.google.com/rss/articles/CBMie0FVX3lxTE9pckZqdmNDanNIakl6SkR2SkZLVWxmREhfNWF6elE2U3YyUG1OQWtGc19CWExiZnJPcURlUWxTS0M3d2ZKdnJFM3E1TENKWE5rTkJYOHhibG5ZRDdDRHBucUVzYUhUUi1MOGNncXNkNXFCdkJCeWtRVm5YZw?oc=5）</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>利多：劳动力短缺限制生产节奏，可能减少短期糖源供应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>斐济</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ChiniMandi称，斐济甘蔗收割受到劳动力短缺拖累。若收割延误持续，糖厂入榨量和生产节奏可能受压。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiekFVX3lxTFBEUUY2QWU3MmxCcjZHcGwzM2phb1gwaG5PRFJEUUFGYVBwRnBjT0lxNzZudk9aODB6MGMzcm9pczNiYmlSbDdTUm5ucUdZTm1HOUFRbWhhazhVYXlvZDNER2NfWkdzb200WDlGY2ZlLUJ6MDdGMktxc2RR?oc=5）</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>利多：收割瓶颈可能削弱甘蔗供应和产糖进度，对糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>印度尼西亚</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ANTARA News称，印尼正推动甘蔗支撑生物乙醇发展，以服务国内乙醇和能源转型目标。若甘蔗制乙醇规模扩大，可能提高糖料需求并影响糖醇分配。来源：ANTARA News（https://news.google.com/rss/articles/CBMinwFBVV95cUxOS1YzTmlmWmFJT1pUYzZMTVZKVUtQUnYzQVhwN2Z1dFI0T3VNUXBaR2cxcFpxNDJqVmw3ejZtY1BIX1RNLUM4VjNtZmZlUzhBNUNHYlFGRk9Fbzh2NW9xaWtTa0hGcGFwdm1rbEh5czNQTEtCc3VhRGZkZ0prSTNaLVVlaFdHMzhUSF9zSlVxSG9yWnV5czBqQUN1dzRNUjTSAZ8BQVVfeXFMTktWM05pZlphSU9aVGM2TE1WSlVLUFJ2M0FYcDdmdXRSNE91TVFwWkdnMXBacTQyalZsN3o2bWNQSF9UTS1DOFYzbWZmZVM4QTVDR2JRRkZPRW84djVvcWlrU2tIRnBhcHZta2xIeXMzUExLQnN1YURmZGdKa0kzWi1VZWhXRzM4VEhfc0pVcUhvclp1eXMwakFDdXc0TVI0?oc=5）</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>利多：甘蔗制乙醇需求增加可能分流部分糖料，对糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>肯尼亚</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>肯尼亚媒体关注一批免税进口糖的来源问题，相关货物流向涉及巴西糖及南非中转。若免税进口增加，将提高肯尼亚国内可用糖源，但也带来贸易监管和原产地核查压力。来源：the-star.co.ke（https://news.google.com/rss/articles/CBMiugFBVV95cUxPa05kUGNibE8ydnd1NWpfRWNPMkZOMTBxQm54OUhla2FLYmJpUnpQUjRkN25LN3ZCbndMZlplT3pNZWNoZzFTQTFOVDd6OHU1RXI0SHg0MC03bjJuWUtSNnpPeU1JRjVYdDNVcFVlVEFZNWM1eU50ZldNWXNROWNJdlBHLWtYSU9ncC1VUUxBUDhrdlZFT042eU82OGpVOGlmc0t5UGtkUnBmaEtpU1RqZjc3dldKcmp5UkE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>利空：进口糖增加补充国内供应，对当地糖价偏利空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>全球</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Barchart指出，原油价格上涨对糖价形成支撑。能源价格走强通常提高乙醇相对吸引力，可能影响甘蔗在制糖和制醇之间的分配。来源：Barchart.com（https://news.google.com/rss/articles/CBMiiAFBVV95cUxQZWFVUFdFYWVLRnlON2YxV2N5YTVKMDdsNFkxVnUtVG5IOHpOMkhDb2xyVTc0TlZlTnIyRm5SV19FU0p2MGFyLTRhVDZFSFN1TFg2bHAySG9hQkFVVjgweGxFLUNnWVJjMWZOa2RDZmVidmVidERiZ1FrakpkaE9mVFlxbnZLa0Zo?oc=5）</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>利多：原油上涨增强乙醇分流预期，对国际糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>波兰拟提高糖税，食品和饮料行业警示相关政策可能增加终端成本。该政策主要影响含糖饮料和加工食品需求，对原糖供应端影响有限。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiswFBVV95cUxOd1QyWVNpQ0FJSkFBSk55NWh1b0pyQzI0NGFGaU5LWGhXSWhlYU16LTdEdnRwM05XVldFNmx2NjV4aFNKeTJ0WHo0cGVqQmJnMUZuXzFfOUpFb1VRckd2Q3VjbDlBaVVXaHl5b19pWEZ6ODhMNGF1LU5aazJjSEFGWk1nektIbGt4SXFxSTFlUXFYWEpEbm9ubWJ5NVJaUkxVOVczU1VxWF9SQko1Mi15ckZiZw?oc=5）</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>中性：税收调整偏向消费端，短期对食糖供需影响有限。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>UkrAgroConsult称，波兰食糖产量可能下降17%。若减产兑现，将收缩当地糖源供应，并增加欧洲区域供应偏紧风险。来源：UkrAgroConsult（https://news.google.com/rss/articles/CBMigwFBVV95cUxNRmgyRnZoMWIyTEUtLUFjS2padHhNR0tuZDE5T0pGTzZLUWlxS1lNQloxaFFUaUpWNW41UEJRUU9RZmR2NUxwY3ViQmx0SVM5cklFM2NHUEt3cUpvekpSM2g1ME1jYXBqZVoza2p4NXphcEFiZlY3Q0hmaVlGRU9xU29DQQ?oc=5）</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>利多：产量下降直接减少供应，对区域糖价偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>美国C&amp;H Sugar在Crockett的罢工线出现逮捕和受伤事件，劳资冲突继续扰动企业运营。若罢工影响炼糖、仓储或发运节奏，可能削弱短期供应稳定性。来源：ABC7 Bay Area（https://news.google.com/rss/articles/CBMilgFBVV95cUxQY2x4cG8yOGF1NTQ3eVBUVW9JRVkzQXBxR25pVEhxRm95UFBEMV9BdEZoVXVocC1uQ0c5TzlmTzREdzRKWUtVbXJQX29zVEY3QkI0TzVCSWktMHRhUE9abU45SlVCVnhzSmdQUkFnMzBpZUtNUUE1eWNSbGVqT01LUkVjb1ZsZ3QteEE2eUR1NV9HLWY2TlHSAZsBQVVfeXFMT0w1bk1yajBVSVp0dlBmMEJOZXlHMUQ5WHgzSEpnYTZack1FVUtsTVYwS2c4TGN0TWtsWktTcjlIemFDTW1OZFNoLUhPcGxWQlJZMGdzVXRjdzBKWVhjZGk5bXMyd01Dd3RXMjJ4R3pwMnNDLWZ2SmVNTjNGUkpGLVg0cWUxTVRpN0pib1lFUUJ3bElLNGU1aDRnWFE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>利多：劳资冲突可能扰动炼糖和物流，对局部供应偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Czapp称，昆士兰甘蔗含糖量提高，抵消了收割开局偏慢的影响。较高糖分有助于提升单位甘蔗产糖效率，缓和收割进度偏慢带来的供应担忧。来源：czapp.com（https://news.google.com/rss/articles/CBMiowFBVV95cUxQcVd5RDJSRzJQX3RzdkhSa2k3TndUSDREUGludzZmaTRlZG1JQ1FxSlNqTzRuc3pSSlVfRk16dTFvOVZtYVpUUFc2aXR1X3A2X3o2RzU3Ul9SODJPdEdMbjlTS2FIMUlnZ1hHM18tTjdTNlVVQU5VWE9PTVNaV1k0S3JSQjAyMnZzYnlZckZmZkxSRnJHUzhQbjdVZ1V4SWFjRlFj?oc=5）</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>利空：甘蔗含糖量改善提高产糖效率，对糖价偏利空。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Thailand cane rainfall news rule
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-22.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-22.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
@@ -636,17 +636,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>英国</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>BBC节目涉及英国甜菜糖厂关闭及农业政策调整，显示英国甜菜糖加工布局继续收缩。相关影响取决于替代工厂承接能力，短期对国内食糖供应仍需跟踪。来源：BBC（https://news.google.com/rss/articles/CBMiUEFVX3lxTE53aXJVWlV3MGE5WEZJRHBhZE8tbm1JbnBvX21HZFJMeG1jaDhjckNBUVM1Q3BJc0VLMWVOcktFbERkbF9vRWlnUDgzdWdzS1lo?oc=5）</t>
+          <t>泰国气象局预报，7月23日06:00至24日06:00，东北部乌隆他尼、孔敬、黎府等核心甘蔗产区有雷阵雨并伴有局地大雨，北部素可泰、彭世洛，中部北碧及东部沙缴、春武里等产区也有雷阵雨。当前处于甘蔗生长阶段，产区降雨有利于补充土壤水分、促进甘蔗生长和单产形成，增加后期食糖供应预期；但官方预报以区域性雷阵雨和局地大雨为主，暂未确认大范围农业损失。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>中性：单厂调整影响区域甜菜消化，但全国供应影响尚不明确。</t>
+          <t>利空，幅度有限：甘蔗生长阶段降雨改善土壤墒情并提高未来糖料供应预期，对糖价利空；但本次以局地雷阵雨为主，影响幅度有限。</t>
         </is>
       </c>
     </row>
@@ -658,12 +658,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The Telegraph称，英国历史最久的糖厂因高能源成本关闭。能源成本上升压缩甜菜糖加工利润，若产能退出落地，可能削弱英国本土制糖能力。来源：The Telegraph（https://news.google.com/rss/articles/CBMiqgFBVV95cUxOa2xFWmhEQmg2M29sUnduS2RtMG41TFJCVDNBNFRuamF2d1NBV09ndGtMLWhnS0dmbXM2eXBNMzJGWE5nTFZtNEJDZjNDbVRNLWk5VzVhc1BiWDlHQXdjTmdZWHVBOGVnQldPcG1PeUVlcTRSZXZjSXExR3phbFVxRlZ3SzI2amtEcEN5aEZnQlZWMTNibXpQVU5vUGhOU2tmTGpNQ3BrSVF6UQ?oc=5）</t>
+          <t>BBC节目涉及英国甜菜糖厂关闭及农业政策调整，显示英国甜菜糖加工布局继续收缩。相关影响取决于替代工厂承接能力，短期对国内食糖供应仍需跟踪。来源：BBC（https://news.google.com/rss/articles/CBMiUEFVX3lxTE53aXJVWlV3MGE5WEZJRHBhZE8tbm1JbnBvX21HZFJMeG1jaDhjckNBUVM1Q3BJc0VLMWVOcktFbERkbF9vRWlnUDgzdWdzS1lo?oc=5）</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>利多：加工产能退出和成本压力可能收缩本土供应，对糖价偏利多。</t>
+          <t>中性：单厂调整影响区域甜菜消化，但全国供应影响尚不明确。</t>
         </is>
       </c>
     </row>
@@ -675,12 +675,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>British Sugar计划关闭Cantley工厂，以提升公司竞争力和运营效率。该调整反映英国甜菜糖行业成本和产能布局压力，但短期供应影响取决于其他工厂承接情况。来源：Food and Drink International（https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR01lb3dWYnZCc0tKWkd5OE42ZjlKa3owRy04ZTA3ZThUcmNid3FmeTd2d0t3N1dXYmQxX0dXcnJjYXo5WmJGd1ctQ3lKZXhtMndYVHhkMkE1YXVWUmZNWEpIZUtYSDBfYmNQZ004bm9jV1JlMW1IWkswa01ralA3eHZ3N0wzZUVhUmhCYkxHNEFCSEMwWFVwT2FBallSZGhGZlY2aXBGTGNkMW5MQVVWclNfQmJEbnFf?oc=5）</t>
+          <t>The Telegraph称，英国历史最久的糖厂因高能源成本关闭。能源成本上升压缩甜菜糖加工利润，若产能退出落地，可能削弱英国本土制糖能力。来源：The Telegraph（https://news.google.com/rss/articles/CBMiqgFBVV95cUxOa2xFWmhEQmg2M29sUnduS2RtMG41TFJCVDNBNFRuamF2d1NBV09ndGtMLWhnS0dmbXM2eXBNMzJGWE5nTFZtNEJDZjNDbVRNLWk5VzVhc1BiWDlHQXdjTmdZWHVBOGVnQldPcG1PeUVlcTRSZXZjSXExR3phbFVxRlZ3SzI2amtEcEN5aEZnQlZWMTNibXpQVU5vUGhOU2tmTGpNQ3BrSVF6UQ?oc=5）</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>中性：产能整合改善企业效率，但对当期供应的影响尚待确认。</t>
+          <t>利多：加工产能退出和成本压力可能收缩本土供应，对糖价偏利多。</t>
         </is>
       </c>
     </row>
@@ -692,29 +692,29 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ChiniMandi称，British Sugar拟关闭历史悠久的Cantley工厂，超过100个岗位面临风险。若关闭执行，将减少当地甜菜加工节点，对区域甜菜收购和制糖能力构成压力。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirAFBVV95cUxObnJJb1pyWU5hbnVUMVBZNHV0MVZ5akZQLTB5RU96OVBkZnhJaEdmV1VyMlY4ZndmTlBBRXB0NFY1bUVScF80YkxUWWhNR1hHWmpLNXFmYndDc1hZTk9IeUk2aEhNYVdkOWsxN2VVTVd1SWVrWDZqOUlEWGdJS3dOR0x4NG5iNDhoRDRoSjJIUmF4a3dIT0hwR3hTVG02UzNrX2xaQ1NHUndTT3VS?oc=5）</t>
+          <t>British Sugar计划关闭Cantley工厂，以提升公司竞争力和运营效率。该调整反映英国甜菜糖行业成本和产能布局压力，但短期供应影响取决于其他工厂承接情况。来源：Food and Drink International（https://news.google.com/rss/articles/CBMiuAFBVV95cUxNR01lb3dWYnZCc0tKWkd5OE42ZjlKa3owRy04ZTA3ZThUcmNid3FmeTd2d0t3N1dXYmQxX0dXcnJjYXo5WmJGd1ctQ3lKZXhtMndYVHhkMkE1YXVWUmZNWEpIZUtYSDBfYmNQZ004bm9jV1JlMW1IWkswa01ralA3eHZ3N0wzZUVhUmhCYkxHNEFCSEMwWFVwT2FBallSZGhGZlY2aXBGTGNkMW5MQVVWclNfQmJEbnFf?oc=5）</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>利多：区域加工能力下降可能削弱本土糖源供给，对糖价偏利多。</t>
+          <t>中性：产能整合改善企业效率，但对当期供应的影响尚待确认。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>斐济</t>
+          <t>英国</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FBC News称，斐济劳动力短缺拖慢食糖生产。采收和压榨环节受限可能影响甘蔗入榨进度，增加当期产糖不确定性。来源：FBC News（https://news.google.com/rss/articles/CBMie0FVX3lxTE9pckZqdmNDanNIakl6SkR2SkZLVWxmREhfNWF6elE2U3YyUG1OQWtGc19CWExiZnJPcURlUWxTS0M3d2ZKdnJFM3E1TENKWE5rTkJYOHhibG5ZRDdDRHBucUVzYUhUUi1MOGNncXNkNXFCdkJCeWtRVm5YZw?oc=5）</t>
+          <t>ChiniMandi称，British Sugar拟关闭历史悠久的Cantley工厂，超过100个岗位面临风险。若关闭执行，将减少当地甜菜加工节点，对区域甜菜收购和制糖能力构成压力。来源：ChiniMandi（https://news.google.com/rss/articles/CBMirAFBVV95cUxObnJJb1pyWU5hbnVUMVBZNHV0MVZ5akZQLTB5RU96OVBkZnhJaEdmV1VyMlY4ZndmTlBBRXB0NFY1bUVScF80YkxUWWhNR1hHWmpLNXFmYndDc1hZTk9IeUk2aEhNYVdkOWsxN2VVTVd1SWVrWDZqOUlEWGdJS3dOR0x4NG5iNDhoRDRoSjJIUmF4a3dIT0hwR3hTVG02UzNrX2xaQ1NHUndTT3VS?oc=5）</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>利多：劳动力短缺限制生产节奏，可能减少短期糖源供应。</t>
+          <t>利多：区域加工能力下降可能削弱本土糖源供给，对糖价偏利多。</t>
         </is>
       </c>
     </row>
@@ -726,80 +726,80 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ChiniMandi称，斐济甘蔗收割受到劳动力短缺拖累。若收割延误持续，糖厂入榨量和生产节奏可能受压。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiekFVX3lxTFBEUUY2QWU3MmxCcjZHcGwzM2phb1gwaG5PRFJEUUFGYVBwRnBjT0lxNzZudk9aODB6MGMzcm9pczNiYmlSbDdTUm5ucUdZTm1HOUFRbWhhazhVYXlvZDNER2NfWkdzb200WDlGY2ZlLUJ6MDdGMktxc2RR?oc=5）</t>
+          <t>FBC News称，斐济劳动力短缺拖慢食糖生产。采收和压榨环节受限可能影响甘蔗入榨进度，增加当期产糖不确定性。来源：FBC News（https://news.google.com/rss/articles/CBMie0FVX3lxTE9pckZqdmNDanNIakl6SkR2SkZLVWxmREhfNWF6elE2U3YyUG1OQWtGc19CWExiZnJPcURlUWxTS0M3d2ZKdnJFM3E1TENKWE5rTkJYOHhibG5ZRDdDRHBucUVzYUhUUi1MOGNncXNkNXFCdkJCeWtRVm5YZw?oc=5）</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>利多：收割瓶颈可能削弱甘蔗供应和产糖进度，对糖价偏利多。</t>
+          <t>利多：劳动力短缺限制生产节奏，可能减少短期糖源供应。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>印度尼西亚</t>
+          <t>斐济</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ANTARA News称，印尼正推动甘蔗支撑生物乙醇发展，以服务国内乙醇和能源转型目标。若甘蔗制乙醇规模扩大，可能提高糖料需求并影响糖醇分配。来源：ANTARA News（https://news.google.com/rss/articles/CBMinwFBVV95cUxOS1YzTmlmWmFJT1pUYzZMTVZKVUtQUnYzQVhwN2Z1dFI0T3VNUXBaR2cxcFpxNDJqVmw3ejZtY1BIX1RNLUM4VjNtZmZlUzhBNUNHYlFGRk9Fbzh2NW9xaWtTa0hGcGFwdm1rbEh5czNQTEtCc3VhRGZkZ0prSTNaLVVlaFdHMzhUSF9zSlVxSG9yWnV5czBqQUN1dzRNUjTSAZ8BQVVfeXFMTktWM05pZlphSU9aVGM2TE1WSlVLUFJ2M0FYcDdmdXRSNE91TVFwWkdnMXBacTQyalZsN3o2bWNQSF9UTS1DOFYzbWZmZVM4QTVDR2JRRkZPRW84djVvcWlrU2tIRnBhcHZta2xIeXMzUExLQnN1YURmZGdKa0kzWi1VZWhXRzM4VEhfc0pVcUhvclp1eXMwakFDdXc0TVI0?oc=5）</t>
+          <t>ChiniMandi称，斐济甘蔗收割受到劳动力短缺拖累。若收割延误持续，糖厂入榨量和生产节奏可能受压。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiekFVX3lxTFBEUUY2QWU3MmxCcjZHcGwzM2phb1gwaG5PRFJEUUFGYVBwRnBjT0lxNzZudk9aODB6MGMzcm9pczNiYmlSbDdTUm5ucUdZTm1HOUFRbWhhazhVYXlvZDNER2NfWkdzb200WDlGY2ZlLUJ6MDdGMktxc2RR?oc=5）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>利多：甘蔗制乙醇需求增加可能分流部分糖料，对糖价偏利多。</t>
+          <t>利多：收割瓶颈可能削弱甘蔗供应和产糖进度，对糖价偏利多。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>肯尼亚</t>
+          <t>印度尼西亚</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>肯尼亚媒体关注一批免税进口糖的来源问题，相关货物流向涉及巴西糖及南非中转。若免税进口增加，将提高肯尼亚国内可用糖源，但也带来贸易监管和原产地核查压力。来源：the-star.co.ke（https://news.google.com/rss/articles/CBMiugFBVV95cUxPa05kUGNibE8ydnd1NWpfRWNPMkZOMTBxQm54OUhla2FLYmJpUnpQUjRkN25LN3ZCbndMZlplT3pNZWNoZzFTQTFOVDd6OHU1RXI0SHg0MC03bjJuWUtSNnpPeU1JRjVYdDNVcFVlVEFZNWM1eU50ZldNWXNROWNJdlBHLWtYSU9ncC1VUUxBUDhrdlZFT042eU82OGpVOGlmc0t5UGtkUnBmaEtpU1RqZjc3dldKcmp5UkE?oc=5）</t>
+          <t>ANTARA News称，印尼正推动甘蔗支撑生物乙醇发展，以服务国内乙醇和能源转型目标。若甘蔗制乙醇规模扩大，可能提高糖料需求并影响糖醇分配。来源：ANTARA News（https://news.google.com/rss/articles/CBMinwFBVV95cUxOS1YzTmlmWmFJT1pUYzZMTVZKVUtQUnYzQVhwN2Z1dFI0T3VNUXBaR2cxcFpxNDJqVmw3ejZtY1BIX1RNLUM4VjNtZmZlUzhBNUNHYlFGRk9Fbzh2NW9xaWtTa0hGcGFwdm1rbEh5czNQTEtCc3VhRGZkZ0prSTNaLVVlaFdHMzhUSF9zSlVxSG9yWnV5czBqQUN1dzRNUjTSAZ8BQVVfeXFMTktWM05pZlphSU9aVGM2TE1WSlVLUFJ2M0FYcDdmdXRSNE91TVFwWkdnMXBacTQyalZsN3o2bWNQSF9UTS1DOFYzbWZmZVM4QTVDR2JRRkZPRW84djVvcWlrU2tIRnBhcHZta2xIeXMzUExLQnN1YURmZGdKa0kzWi1VZWhXRzM4VEhfc0pVcUhvclp1eXMwakFDdXc0TVI0?oc=5）</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>利空：进口糖增加补充国内供应，对当地糖价偏利空。</t>
+          <t>利多：甘蔗制乙醇需求增加可能分流部分糖料，对糖价偏利多。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>全球</t>
+          <t>肯尼亚</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Barchart指出，原油价格上涨对糖价形成支撑。能源价格走强通常提高乙醇相对吸引力，可能影响甘蔗在制糖和制醇之间的分配。来源：Barchart.com（https://news.google.com/rss/articles/CBMiiAFBVV95cUxQZWFVUFdFYWVLRnlON2YxV2N5YTVKMDdsNFkxVnUtVG5IOHpOMkhDb2xyVTc0TlZlTnIyRm5SV19FU0p2MGFyLTRhVDZFSFN1TFg2bHAySG9hQkFVVjgweGxFLUNnWVJjMWZOa2RDZmVidmVidERiZ1FrakpkaE9mVFlxbnZLa0Zo?oc=5）</t>
+          <t>肯尼亚媒体关注一批免税进口糖的来源问题，相关货物流向涉及巴西糖及南非中转。若免税进口增加，将提高肯尼亚国内可用糖源，但也带来贸易监管和原产地核查压力。来源：the-star.co.ke（https://news.google.com/rss/articles/CBMiugFBVV95cUxPa05kUGNibE8ydnd1NWpfRWNPMkZOMTBxQm54OUhla2FLYmJpUnpQUjRkN25LN3ZCbndMZlplT3pNZWNoZzFTQTFOVDd6OHU1RXI0SHg0MC03bjJuWUtSNnpPeU1JRjVYdDNVcFVlVEFZNWM1eU50ZldNWXNROWNJdlBHLWtYSU9ncC1VUUxBUDhrdlZFT042eU82OGpVOGlmc0t5UGtkUnBmaEtpU1RqZjc3dldKcmp5UkE?oc=5）</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>利多：原油上涨增强乙醇分流预期，对国际糖价偏利多。</t>
+          <t>利空：进口糖增加补充国内供应，对当地糖价偏利空。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>波兰</t>
+          <t>全球</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>波兰拟提高糖税，食品和饮料行业警示相关政策可能增加终端成本。该政策主要影响含糖饮料和加工食品需求，对原糖供应端影响有限。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiswFBVV95cUxOd1QyWVNpQ0FJSkFBSk55NWh1b0pyQzI0NGFGaU5LWGhXSWhlYU16LTdEdnRwM05XVldFNmx2NjV4aFNKeTJ0WHo0cGVqQmJnMUZuXzFfOUpFb1VRckd2Q3VjbDlBaVVXaHl5b19pWEZ6ODhMNGF1LU5aazJjSEFGWk1nektIbGt4SXFxSTFlUXFYWEpEbm9ubWJ5NVJaUkxVOVczU1VxWF9SQko1Mi15ckZiZw?oc=5）</t>
+          <t>Barchart指出，原油价格上涨对糖价形成支撑。能源价格走强通常提高乙醇相对吸引力，可能影响甘蔗在制糖和制醇之间的分配。来源：Barchart.com（https://news.google.com/rss/articles/CBMiiAFBVV95cUxQZWFVUFdFYWVLRnlON2YxV2N5YTVKMDdsNFkxVnUtVG5IOHpOMkhDb2xyVTc0TlZlTnIyRm5SV19FU0p2MGFyLTRhVDZFSFN1TFg2bHAySG9hQkFVVjgweGxFLUNnWVJjMWZOa2RDZmVidmVidERiZ1FrakpkaE9mVFlxbnZLa0Zo?oc=5）</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>中性：税收调整偏向消费端，短期对食糖供需影响有限。</t>
+          <t>利多：原油上涨增强乙醇分流预期，对国际糖价偏利多。</t>
         </is>
       </c>
     </row>
@@ -811,44 +811,61 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>UkrAgroConsult称，波兰食糖产量可能下降17%。若减产兑现，将收缩当地糖源供应，并增加欧洲区域供应偏紧风险。来源：UkrAgroConsult（https://news.google.com/rss/articles/CBMigwFBVV95cUxNRmgyRnZoMWIyTEUtLUFjS2padHhNR0tuZDE5T0pGTzZLUWlxS1lNQloxaFFUaUpWNW41UEJRUU9RZmR2NUxwY3ViQmx0SVM5cklFM2NHUEt3cUpvekpSM2g1ME1jYXBqZVoza2p4NXphcEFiZlY3Q0hmaVlGRU9xU29DQQ?oc=5）</t>
+          <t>波兰拟提高糖税，食品和饮料行业警示相关政策可能增加终端成本。该政策主要影响含糖饮料和加工食品需求，对原糖供应端影响有限。来源：ChiniMandi（https://news.google.com/rss/articles/CBMiswFBVV95cUxOd1QyWVNpQ0FJSkFBSk55NWh1b0pyQzI0NGFGaU5LWGhXSWhlYU16LTdEdnRwM05XVldFNmx2NjV4aFNKeTJ0WHo0cGVqQmJnMUZuXzFfOUpFb1VRckd2Q3VjbDlBaVVXaHl5b19pWEZ6ODhMNGF1LU5aazJjSEFGWk1nektIbGt4SXFxSTFlUXFYWEpEbm9ubWJ5NVJaUkxVOVczU1VxWF9SQko1Mi15ckZiZw?oc=5）</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>利多：产量下降直接减少供应，对区域糖价偏利多。</t>
+          <t>中性：税收调整偏向消费端，短期对食糖供需影响有限。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>美国</t>
+          <t>波兰</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>美国C&amp;H Sugar在Crockett的罢工线出现逮捕和受伤事件，劳资冲突继续扰动企业运营。若罢工影响炼糖、仓储或发运节奏，可能削弱短期供应稳定性。来源：ABC7 Bay Area（https://news.google.com/rss/articles/CBMilgFBVV95cUxQY2x4cG8yOGF1NTQ3eVBUVW9JRVkzQXBxR25pVEhxRm95UFBEMV9BdEZoVXVocC1uQ0c5TzlmTzREdzRKWUtVbXJQX29zVEY3QkI0TzVCSWktMHRhUE9abU45SlVCVnhzSmdQUkFnMzBpZUtNUUE1eWNSbGVqT01LUkVjb1ZsZ3QteEE2eUR1NV9HLWY2TlHSAZsBQVVfeXFMT0w1bk1yajBVSVp0dlBmMEJOZXlHMUQ5WHgzSEpnYTZack1FVUtsTVYwS2c4TGN0TWtsWktTcjlIemFDTW1OZFNoLUhPcGxWQlJZMGdzVXRjdzBKWVhjZGk5bXMyd01Dd3RXMjJ4R3pwMnNDLWZ2SmVNTjNGUkpGLVg0cWUxTVRpN0pib1lFUUJ3bElLNGU1aDRnWFE?oc=5）</t>
+          <t>UkrAgroConsult称，波兰食糖产量可能下降17%。若减产兑现，将收缩当地糖源供应，并增加欧洲区域供应偏紧风险。来源：UkrAgroConsult（https://news.google.com/rss/articles/CBMigwFBVV95cUxNRmgyRnZoMWIyTEUtLUFjS2padHhNR0tuZDE5T0pGTzZLUWlxS1lNQloxaFFUaUpWNW41UEJRUU9RZmR2NUxwY3ViQmx0SVM5cklFM2NHUEt3cUpvekpSM2g1ME1jYXBqZVoza2p4NXphcEFiZlY3Q0hmaVlGRU9xU29DQQ?oc=5）</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>利多：劳资冲突可能扰动炼糖和物流，对局部供应偏利多。</t>
+          <t>利多：产量下降直接减少供应，对区域糖价偏利多。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>美国C&amp;H Sugar在Crockett的罢工线出现逮捕和受伤事件，劳资冲突继续扰动企业运营。若罢工影响炼糖、仓储或发运节奏，可能削弱短期供应稳定性。来源：ABC7 Bay Area（https://news.google.com/rss/articles/CBMilgFBVV95cUxQY2x4cG8yOGF1NTQ3eVBUVW9JRVkzQXBxR25pVEhxRm95UFBEMV9BdEZoVXVocC1uQ0c5TzlmTzREdzRKWUtVbXJQX29zVEY3QkI0TzVCSWktMHRhUE9abU45SlVCVnhzSmdQUkFnMzBpZUtNUUE1eWNSbGVqT01LUkVjb1ZsZ3QteEE2eUR1NV9HLWY2TlHSAZsBQVVfeXFMT0w1bk1yajBVSVp0dlBmMEJOZXlHMUQ5WHgzSEpnYTZack1FVUtsTVYwS2c4TGN0TWtsWktTcjlIemFDTW1OZFNoLUhPcGxWQlJZMGdzVXRjdzBKWVhjZGk5bXMyd01Dd3RXMjJ4R3pwMnNDLWZ2SmVNTjNGUkpGLVg0cWUxTVRpN0pib1lFUUJ3bElLNGU1aDRnWFE?oc=5）</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>利多：劳资冲突可能扰动炼糖和物流，对局部供应偏利多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>澳大利亚</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Czapp称，昆士兰甘蔗含糖量提高，抵消了收割开局偏慢的影响。较高糖分有助于提升单位甘蔗产糖效率，缓和收割进度偏慢带来的供应担忧。来源：czapp.com（https://news.google.com/rss/articles/CBMiowFBVV95cUxQcVd5RDJSRzJQX3RzdkhSa2k3TndUSDREUGludzZmaTRlZG1JQ1FxSlNqTzRuc3pSSlVfRk16dTFvOVZtYVpUUFc2aXR1X3A2X3o2RzU3Ul9SODJPdEdMbjlTS2FIMUlnZ1hHM18tTjdTNlVVQU5VWE9PTVNaV1k0S3JSQjAyMnZzYnlZckZmZkxSRnJHUzhQbjdVZ1V4SWFjRlFj?oc=5）</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>利空：甘蔗含糖量改善提高产糖效率，对糖价偏利空。</t>
         </is>

</xml_diff>

<commit_message>
Revise Thailand rainfall impact rule
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-22.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-22.xlsx
@@ -641,12 +641,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>泰国气象局预报，7月23日06:00至24日06:00，东北部乌隆他尼、孔敬、黎府等核心甘蔗产区有雷阵雨并伴有局地大雨，北部素可泰、彭世洛，中部北碧及东部沙缴、春武里等产区也有雷阵雨。当前处于甘蔗生长阶段，产区降雨有利于补充土壤水分、促进甘蔗生长和单产形成，增加后期食糖供应预期；但官方预报以区域性雷阵雨和局地大雨为主，暂未确认大范围农业损失。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
+          <t>泰国气象局预报，7月23日06:00至24日06:00，东北部乌隆他尼、孔敬、黎府等核心甘蔗产区有雷阵雨并伴有局地大雨，北部素可泰、彭世洛，中部北碧及东部沙缴、春武里等产区也有雷阵雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>利空，幅度有限：甘蔗生长阶段降雨改善土壤墒情并提高未来糖料供应预期，对糖价利空；但本次以局地雷阵雨为主，影响幅度有限。</t>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>

</xml_diff>